<commit_message>
changes for computer gold
</commit_message>
<xml_diff>
--- a/uploads/sandbox_ComputerGold_excel.xlsx
+++ b/uploads/sandbox_ComputerGold_excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hanna\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75A8171C-1099-40E9-B393-2E9426EB21A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87D85A82-5255-46CC-B3AE-16141FA44160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{760F17F9-C6B3-41C5-B918-0FB8C401C1FD}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="939" uniqueCount="729">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="937" uniqueCount="727">
   <si>
     <t>sellerBusinessName</t>
   </si>
@@ -2214,16 +2214,10 @@
     <t>PO#</t>
   </si>
   <si>
+    <t>(Delivery Challan Number / Date)</t>
+  </si>
+  <si>
     <t>134 / 08-07-2025</t>
-  </si>
-  <si>
-    <t>132 / 08-07-2025</t>
-  </si>
-  <si>
-    <t>Enter Delivery Challan Number Here</t>
-  </si>
-  <si>
-    <t>Enter Puchase Order Number here</t>
   </si>
 </sst>
 </file>
@@ -2877,12 +2871,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80E7F905-168E-44F5-986A-893891B51600}">
-  <dimension ref="A1:S28"/>
+  <dimension ref="A1:S27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="24.5546875" style="1" customWidth="1"/>
-    <col min="3" max="4" width="13.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" style="1"/>
+    <col min="4" max="4" width="13.33203125" style="1" customWidth="1"/>
     <col min="5" max="5" width="11.6640625" style="1" customWidth="1"/>
     <col min="6" max="6" width="11.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="20.109375" style="1" customWidth="1"/>
@@ -2990,10 +2985,10 @@
         <v>724</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>726</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>725</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>728</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="18" x14ac:dyDescent="0.35">
@@ -3059,12 +3054,6 @@
       <c r="A23" s="4" t="s">
         <v>722</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>726</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>727</v>
-      </c>
     </row>
     <row r="24" spans="1:18" ht="18" x14ac:dyDescent="0.35">
       <c r="A24" s="3"/>
@@ -3173,9 +3162,6 @@
       <c r="Q27" s="1" t="s">
         <v>721</v>
       </c>
-    </row>
-    <row r="28" spans="1:18" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>